<commit_message>
Component fractional dataset generated using simulation
</commit_message>
<xml_diff>
--- a/data/asm2d-tsn/asm2d_tsn_workbook.xlsx
+++ b/data/asm2d-tsn/asm2d_tsn_workbook.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eselerio\projects\pibre-model\data\asm2d-tsn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE39B76-AAE6-4F8B-B81C-27576AE36217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314CE22D-09F0-44EF-9AED-E4DD7ACA0B39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="250">
   <si>
     <t>process_index</t>
   </si>
@@ -199,18 +199,6 @@
   </si>
   <si>
     <t>unit</t>
-  </si>
-  <si>
-    <t>COD</t>
-  </si>
-  <si>
-    <t>TN</t>
-  </si>
-  <si>
-    <t>TP</t>
-  </si>
-  <si>
-    <t>TSS</t>
   </si>
   <si>
     <t>Dissolved</t>
@@ -2171,16 +2159,33 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:W21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="4" width="12" customWidth="1"/>
-    <col min="5" max="7" width="26" customWidth="1"/>
+    <col min="1" max="1" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.08984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="3.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="5.7265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="3.36328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="3.7265625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="4.08984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="6.36328125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="21" max="22" width="6.54296875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="8.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>50</v>
       </c>
@@ -2190,404 +2195,1484 @@
       <c r="C1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" t="s">
+        <v>9</v>
+      </c>
+      <c r="L1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" t="s">
+        <v>16</v>
+      </c>
+      <c r="S1" t="s">
+        <v>17</v>
+      </c>
+      <c r="T1" t="s">
+        <v>18</v>
+      </c>
+      <c r="U1" t="s">
+        <v>19</v>
+      </c>
+      <c r="V1" t="s">
+        <v>20</v>
+      </c>
+      <c r="W1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>53</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>57</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+        <v>54</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2">
+        <v>0</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D3">
-        <f>1</f>
+        <v>0</v>
+      </c>
+      <c r="E3">
         <v>1</v>
       </c>
-      <c r="E3">
-        <f>parameter_table!$E$11</f>
-        <v>0</v>
-      </c>
       <c r="F3">
-        <f>parameter_table!$E$16</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3">
+        <v>0</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D4">
-        <f>1</f>
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>56</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
       </c>
       <c r="E5">
-        <f>1</f>
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>0</v>
+      </c>
+      <c r="U5">
+        <v>0</v>
+      </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>56</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
       </c>
       <c r="E6">
-        <f>1</f>
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <v>0</v>
+      </c>
+      <c r="U6">
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <v>0</v>
+      </c>
+      <c r="W6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>56</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
       </c>
       <c r="E7">
-        <f>1</f>
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>0</v>
+      </c>
+      <c r="U7">
+        <v>0</v>
+      </c>
+      <c r="V7">
+        <v>0</v>
+      </c>
+      <c r="W7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <v>0</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <v>0</v>
+      </c>
+      <c r="U8">
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <v>0</v>
+      </c>
+      <c r="W8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>57</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
       </c>
       <c r="F9">
-        <f>1</f>
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+      <c r="K9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
+      <c r="R9">
+        <v>0</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
+      <c r="T9">
+        <v>0</v>
+      </c>
+      <c r="U9">
+        <v>0</v>
+      </c>
+      <c r="V9">
+        <v>0</v>
+      </c>
+      <c r="W9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
         <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D10">
-        <f>1</f>
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10">
         <v>1</v>
       </c>
-      <c r="E10">
-        <f>parameter_table!$E$10</f>
-        <v>0.01</v>
-      </c>
-      <c r="F10">
-        <f>parameter_table!$E$15</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>0</v>
+      </c>
+      <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
+        <v>0</v>
+      </c>
+      <c r="W10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>1</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11">
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <v>0</v>
+      </c>
+      <c r="U11">
+        <v>0</v>
+      </c>
+      <c r="V11">
+        <v>0</v>
+      </c>
+      <c r="W11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>
       </c>
       <c r="C12" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12">
+        <v>1</v>
+      </c>
+      <c r="O12">
+        <v>0</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <v>0</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <v>0</v>
+      </c>
+      <c r="U12">
+        <v>0</v>
+      </c>
+      <c r="V12">
+        <v>0</v>
+      </c>
+      <c r="W12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>59</v>
-      </c>
-      <c r="D12">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="E12">
-        <f>parameter_table!$E$12</f>
-        <v>0.02</v>
-      </c>
-      <c r="F12">
-        <f>parameter_table!$E$17</f>
-        <v>0.01</v>
-      </c>
-      <c r="G12">
-        <f>parameter_table!$E$20</f>
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>63</v>
       </c>
       <c r="B13" t="s">
         <v>13</v>
       </c>
       <c r="C13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13">
+        <v>1</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <v>0</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13">
+        <v>0</v>
+      </c>
+      <c r="T13">
+        <v>0</v>
+      </c>
+      <c r="U13">
+        <v>0</v>
+      </c>
+      <c r="V13">
+        <v>0</v>
+      </c>
+      <c r="W13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
         <v>59</v>
-      </c>
-      <c r="D13">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="E13">
-        <f>parameter_table!$E$13</f>
-        <v>0</v>
-      </c>
-      <c r="F13">
-        <f>parameter_table!$E$18</f>
-        <v>0</v>
-      </c>
-      <c r="G13">
-        <f>parameter_table!$E$21</f>
-        <v>0.75</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>63</v>
       </c>
       <c r="B14" t="s">
         <v>14</v>
       </c>
       <c r="C14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+      <c r="K14">
+        <v>0</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>0</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>0</v>
+      </c>
+      <c r="P14">
+        <v>1</v>
+      </c>
+      <c r="Q14">
+        <v>0</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14">
+        <v>0</v>
+      </c>
+      <c r="T14">
+        <v>0</v>
+      </c>
+      <c r="U14">
+        <v>0</v>
+      </c>
+      <c r="V14">
+        <v>0</v>
+      </c>
+      <c r="W14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
         <v>59</v>
-      </c>
-      <c r="D14">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="E14">
-        <f>parameter_table!$E$14</f>
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="F14">
-        <f>parameter_table!$E$19</f>
-        <v>0.02</v>
-      </c>
-      <c r="G14">
-        <f>parameter_table!$E$22</f>
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>63</v>
       </c>
       <c r="B15" t="s">
         <v>15</v>
       </c>
       <c r="C15" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>0</v>
+      </c>
+      <c r="K15">
+        <v>0</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>1</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15">
+        <v>0</v>
+      </c>
+      <c r="T15">
+        <v>0</v>
+      </c>
+      <c r="U15">
+        <v>0</v>
+      </c>
+      <c r="V15">
+        <v>0</v>
+      </c>
+      <c r="W15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>59</v>
-      </c>
-      <c r="D15">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="E15">
-        <f>parameter_table!$E$14</f>
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="F15">
-        <f>parameter_table!$E$19</f>
-        <v>0.02</v>
-      </c>
-      <c r="G15">
-        <f>parameter_table!$E$22</f>
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>63</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
       </c>
       <c r="C16" t="s">
-        <v>61</v>
+        <v>57</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>0</v>
       </c>
       <c r="F16">
-        <f>1</f>
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>0</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16">
+        <v>0</v>
+      </c>
+      <c r="N16">
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <v>0</v>
+      </c>
+      <c r="R16">
         <v>1</v>
       </c>
-      <c r="G16">
-        <f>parameter_table!$E$24</f>
-        <v>3.23</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="S16">
+        <v>0</v>
+      </c>
+      <c r="T16">
+        <v>0</v>
+      </c>
+      <c r="U16">
+        <v>0</v>
+      </c>
+      <c r="V16">
+        <v>0</v>
+      </c>
+      <c r="W16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B17" t="s">
         <v>17</v>
       </c>
       <c r="C17" t="s">
+        <v>55</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>0</v>
+      </c>
+      <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <v>0</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17">
+        <v>1</v>
+      </c>
+      <c r="T17">
+        <v>0</v>
+      </c>
+      <c r="U17">
+        <v>0</v>
+      </c>
+      <c r="V17">
+        <v>0</v>
+      </c>
+      <c r="W17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>59</v>
-      </c>
-      <c r="D17">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="G17">
-        <f>parameter_table!$E$23</f>
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>63</v>
       </c>
       <c r="B18" t="s">
         <v>18</v>
       </c>
       <c r="C18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>0</v>
+      </c>
+      <c r="N18">
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="P18">
+        <v>0</v>
+      </c>
+      <c r="Q18">
+        <v>0</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+      <c r="S18">
+        <v>0</v>
+      </c>
+      <c r="T18">
+        <v>1</v>
+      </c>
+      <c r="U18">
+        <v>0</v>
+      </c>
+      <c r="V18">
+        <v>0</v>
+      </c>
+      <c r="W18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>59</v>
-      </c>
-      <c r="D18">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="E18">
-        <f>parameter_table!$E$14</f>
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="F18">
-        <f>parameter_table!$E$19</f>
-        <v>0.02</v>
-      </c>
-      <c r="G18">
-        <f>parameter_table!$E$22</f>
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>63</v>
       </c>
       <c r="B19" t="s">
         <v>19</v>
       </c>
       <c r="C19" t="s">
+        <v>55</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>0</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>0</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <v>0</v>
+      </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19">
+        <v>0</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <v>0</v>
+      </c>
+      <c r="T19">
+        <v>0</v>
+      </c>
+      <c r="U19">
+        <v>1</v>
+      </c>
+      <c r="V19">
+        <v>0</v>
+      </c>
+      <c r="W19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>59</v>
-      </c>
-      <c r="D19">
-        <f>1</f>
-        <v>1</v>
-      </c>
-      <c r="E19">
-        <f>parameter_table!$E$14</f>
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="F19">
-        <f>parameter_table!$E$19</f>
-        <v>0.02</v>
-      </c>
-      <c r="G19">
-        <f>parameter_table!$E$22</f>
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>63</v>
       </c>
       <c r="B20" t="s">
         <v>20</v>
       </c>
       <c r="C20" t="s">
-        <v>64</v>
+        <v>60</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
       </c>
       <c r="F20">
-        <f>parameter_table!$E$25</f>
-        <v>0.20499999999999999</v>
+        <v>0</v>
       </c>
       <c r="G20">
-        <f>1</f>
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
+      </c>
+      <c r="M20">
+        <v>0</v>
+      </c>
+      <c r="N20">
+        <v>0</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
+        <v>0</v>
+      </c>
+      <c r="R20">
+        <v>0</v>
+      </c>
+      <c r="S20">
+        <v>0</v>
+      </c>
+      <c r="T20">
+        <v>0</v>
+      </c>
+      <c r="U20">
+        <v>0</v>
+      </c>
+      <c r="V20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="W20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B21" t="s">
         <v>21</v>
       </c>
       <c r="C21" t="s">
-        <v>64</v>
+        <v>60</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
       </c>
       <c r="G21">
-        <f>1</f>
+        <v>0</v>
+      </c>
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>0</v>
+      </c>
+      <c r="L21">
+        <v>0</v>
+      </c>
+      <c r="M21">
+        <v>0</v>
+      </c>
+      <c r="N21">
+        <v>0</v>
+      </c>
+      <c r="O21">
+        <v>0</v>
+      </c>
+      <c r="P21">
+        <v>0</v>
+      </c>
+      <c r="Q21">
+        <v>0</v>
+      </c>
+      <c r="R21">
+        <v>0</v>
+      </c>
+      <c r="S21">
+        <v>0</v>
+      </c>
+      <c r="T21">
+        <v>0</v>
+      </c>
+      <c r="U21">
+        <v>0</v>
+      </c>
+      <c r="V21">
+        <v>0</v>
+      </c>
+      <c r="W21">
         <v>1</v>
       </c>
     </row>
@@ -2614,19 +3699,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>65</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>52</v>
@@ -2634,1622 +3719,1622 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E2" s="3">
         <v>0.625</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" t="s">
         <v>70</v>
       </c>
-      <c r="B3" t="s">
-        <v>74</v>
-      </c>
       <c r="C3" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D3" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="E3" s="4">
         <v>0.625</v>
       </c>
       <c r="F3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B4" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C4" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="D4" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E4" s="4">
         <v>0.2</v>
       </c>
       <c r="F4" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C5" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D5" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E5" s="4">
         <v>0.4</v>
       </c>
       <c r="F5" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="D6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E6" s="4">
         <v>0.18</v>
       </c>
       <c r="F6" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B7" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C7" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="D7" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E7" s="4">
         <v>0.08</v>
       </c>
       <c r="F7" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B8" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C8" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D8" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E8" s="4">
         <v>0</v>
       </c>
       <c r="F8" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B9" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C9" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="D9" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E9" s="4">
         <v>0.1</v>
       </c>
       <c r="F9" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E10" s="3">
         <v>0.01</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>87</v>
+      </c>
+      <c r="B11" t="s">
         <v>91</v>
       </c>
-      <c r="B11" t="s">
-        <v>95</v>
-      </c>
       <c r="C11" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="D11" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E11" s="4">
         <v>0</v>
       </c>
       <c r="F11" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B12" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="C12" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D12" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E12" s="4">
         <v>0.02</v>
       </c>
       <c r="F12" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B13" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="C13" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D13" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E13" s="4">
         <v>0</v>
       </c>
       <c r="F13" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B14" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C14" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D14" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E14" s="4">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F14" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B15" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C15" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D15" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="E15" s="4">
         <v>0</v>
       </c>
       <c r="F15" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B16" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C16" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D16" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="E16" s="4">
         <v>0</v>
       </c>
       <c r="F16" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B17" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C17" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="D17" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="E17" s="4">
         <v>0.01</v>
       </c>
       <c r="F17" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B18" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C18" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="D18" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E18" s="4">
         <v>0</v>
       </c>
       <c r="F18" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B19" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="C19" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D19" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E19" s="4">
         <v>0.02</v>
       </c>
       <c r="F19" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B20" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="C20" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="D20" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E20" s="4">
         <v>0.75</v>
       </c>
       <c r="F20" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B21" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C21" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D21" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E21" s="4">
         <v>0.75</v>
       </c>
       <c r="F21" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B22" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C22" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D22" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="E22" s="4">
         <v>0.9</v>
       </c>
       <c r="F22" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B23" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C23" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D23" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E23" s="4">
         <v>0.6</v>
       </c>
       <c r="F23" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B24" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C24" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D24" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="E24" s="4">
         <v>3.23</v>
       </c>
       <c r="F24" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B25" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C25" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D25" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E25" s="4">
         <v>0.20499999999999999</v>
       </c>
       <c r="F25" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="E26" s="3">
         <v>3</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
+        <v>124</v>
+      </c>
+      <c r="B27" t="s">
         <v>128</v>
       </c>
-      <c r="B27" t="s">
-        <v>132</v>
-      </c>
       <c r="C27" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D27" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="E27" s="4">
         <v>0.6</v>
       </c>
       <c r="F27" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B28" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C28" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D28" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="E28" s="4">
         <v>0.6</v>
       </c>
       <c r="F28" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B29" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C29" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D29" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E29" s="4">
         <v>0.4</v>
       </c>
       <c r="F29" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B30" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C30" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="D30" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E30" s="4">
         <v>0.2</v>
       </c>
       <c r="F30" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B31" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="C31" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D31" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E31" s="4">
         <v>0.5</v>
       </c>
       <c r="F31" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B32" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C32" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D32" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="E32" s="4">
         <v>0.5</v>
       </c>
       <c r="F32" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B33" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="C33" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D33" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="E33" s="4">
         <v>0.5</v>
       </c>
       <c r="F33" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B34" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="C34" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D34" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="E34" s="4">
         <v>0.1</v>
       </c>
       <c r="F34" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="E35" s="3">
         <v>6</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
+        <v>146</v>
+      </c>
+      <c r="B36" t="s">
+        <v>149</v>
+      </c>
+      <c r="C36" t="s">
+        <v>149</v>
+      </c>
+      <c r="D36" t="s">
         <v>150</v>
-      </c>
-      <c r="B36" t="s">
-        <v>153</v>
-      </c>
-      <c r="C36" t="s">
-        <v>153</v>
-      </c>
-      <c r="D36" t="s">
-        <v>154</v>
       </c>
       <c r="E36" s="4">
         <v>3</v>
       </c>
       <c r="F36" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B37" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="C37" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D37" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="E37" s="4">
         <v>0.9</v>
       </c>
       <c r="F37" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B38" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C38" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="D38" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="E38" s="4">
         <v>0.9</v>
       </c>
       <c r="F38" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B39" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C39" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="D39" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="E39" s="4">
         <v>0.4</v>
       </c>
       <c r="F39" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B40" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C40" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="D40" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="E40" s="4">
         <v>0.2</v>
       </c>
       <c r="F40" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B41" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="C41" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="D41" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="E41" s="4">
         <v>4</v>
       </c>
       <c r="F41" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B42" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="C42" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="D42" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E42" s="4">
         <v>4</v>
       </c>
       <c r="F42" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B43" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C43" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="D43" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E43" s="4">
         <v>4</v>
       </c>
       <c r="F43" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B44" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C44" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="D44" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E44" s="4">
         <v>0.5</v>
       </c>
       <c r="F44" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B45" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="C45" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="D45" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="E45" s="4">
         <v>0.5</v>
       </c>
       <c r="F45" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B46" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C46" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="D46" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="E46" s="4">
         <v>0.5</v>
       </c>
       <c r="F46" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B47" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C47" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="D47" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="E47" s="4">
         <v>0.05</v>
       </c>
       <c r="F47" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B48" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C48" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D48" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="E48" s="4">
         <v>0.01</v>
       </c>
       <c r="F48" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B49" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C49" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D49" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E49" s="4">
         <v>0.1</v>
       </c>
       <c r="F49" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="E50" s="3">
         <v>5</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
+        <v>178</v>
+      </c>
+      <c r="B51" t="s">
+        <v>181</v>
+      </c>
+      <c r="C51" t="s">
+        <v>181</v>
+      </c>
+      <c r="D51" t="s">
         <v>182</v>
-      </c>
-      <c r="B51" t="s">
-        <v>185</v>
-      </c>
-      <c r="C51" t="s">
-        <v>185</v>
-      </c>
-      <c r="D51" t="s">
-        <v>186</v>
       </c>
       <c r="E51" s="4">
         <v>0.6</v>
       </c>
       <c r="F51" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B52" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="C52" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D52" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E52" s="4">
         <v>0.56000000000000005</v>
       </c>
       <c r="F52" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B53" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C53" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D53" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="E53" s="4">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F53" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B54" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C54" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="D54" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="E54" s="4">
         <v>0.9</v>
       </c>
       <c r="F54" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B55" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C55" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="D55" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="E55" s="4">
         <v>0.2</v>
       </c>
       <c r="F55" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B56" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="C56" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="D56" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="E56" s="4">
         <v>0.2</v>
       </c>
       <c r="F56" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B57" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C57" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="D57" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="E57" s="4">
         <v>0.2</v>
       </c>
       <c r="F57" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B58" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C58" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="D58" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="E58" s="4">
         <v>0.2</v>
       </c>
       <c r="F58" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B59" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C59" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="D59" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="E59" s="4">
         <v>0.5</v>
       </c>
       <c r="F59" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B60" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C60" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="D60" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="E60" s="4">
         <v>0.5</v>
       </c>
       <c r="F60" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B61" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="C61" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="D61" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="E61" s="4">
         <v>0.5</v>
       </c>
       <c r="F61" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B62" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="C62" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D62" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="E62" s="4">
         <v>0.05</v>
       </c>
       <c r="F62" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B63" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C63" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D63" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="E63" s="4">
         <v>0.2</v>
       </c>
       <c r="F63" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B64" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C64" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="D64" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="E64" s="4">
         <v>0.01</v>
       </c>
       <c r="F64" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B65" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="C65" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="D65" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="E65" s="4">
         <v>0.1</v>
       </c>
       <c r="F65" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B66" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="C66" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="D66" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="E66" s="4">
         <v>0.01</v>
       </c>
       <c r="F66" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B67" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="C67" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="D67" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="E67" s="4">
         <v>0.34</v>
       </c>
       <c r="F67" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B68" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="C68" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="D68" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="E68" s="4">
         <v>0.02</v>
       </c>
       <c r="F68" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B69" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="C69" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="D69" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="E69" s="4">
         <v>0.01</v>
       </c>
       <c r="F69" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="E70" s="3">
         <v>1.81</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
+        <v>221</v>
+      </c>
+      <c r="B71" t="s">
+        <v>224</v>
+      </c>
+      <c r="C71" t="s">
+        <v>224</v>
+      </c>
+      <c r="D71" t="s">
         <v>225</v>
-      </c>
-      <c r="B71" t="s">
-        <v>228</v>
-      </c>
-      <c r="C71" t="s">
-        <v>228</v>
-      </c>
-      <c r="D71" t="s">
-        <v>229</v>
       </c>
       <c r="E71" s="4">
         <v>1.52</v>
       </c>
       <c r="F71" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B72" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="C72" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="D72" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="E72" s="4">
         <v>0.2</v>
       </c>
       <c r="F72" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B73" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="C73" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="D73" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="E73" s="4">
         <v>0.17</v>
       </c>
       <c r="F73" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B74" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="C74" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="D74" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="E74" s="4">
         <v>0.74</v>
       </c>
       <c r="F74" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B75" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="C75" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="D75" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="E75" s="4">
         <v>1.75</v>
       </c>
       <c r="F75" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B76" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C76" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="D76" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="E76" s="4">
         <v>0.5</v>
       </c>
       <c r="F76" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B77" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="C77" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="D77" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="E77" s="4">
         <v>0.5</v>
       </c>
       <c r="F77" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B78" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="C78" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="D78" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="E78" s="4">
         <v>0.5</v>
       </c>
       <c r="F78" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B79" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="C79" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="D79" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="E79" s="4">
         <v>0.01</v>
       </c>
       <c r="F79" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="E80" s="3">
         <v>1</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
+        <v>242</v>
+      </c>
+      <c r="B81" t="s">
         <v>246</v>
       </c>
-      <c r="B81" t="s">
-        <v>250</v>
-      </c>
       <c r="C81" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="D81" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="E81" s="4">
         <v>0.6</v>
       </c>
       <c r="F81" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="B82" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="C82" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="D82" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="E82" s="4">
         <v>0.5</v>
       </c>
       <c r="F82" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Made xomposite calculation exogenous and fractional components the only input and outputs of all models
</commit_message>
<xml_diff>
--- a/data/asm2d-tsn/asm2d_tsn_workbook.xlsx
+++ b/data/asm2d-tsn/asm2d_tsn_workbook.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eselerio\projects\pibre-model\data\asm2d-tsn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{314CE22D-09F0-44EF-9AED-E4DD7ACA0B39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE39B76-AAE6-4F8B-B81C-27576AE36217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="254">
   <si>
     <t>process_index</t>
   </si>
@@ -199,6 +199,18 @@
   </si>
   <si>
     <t>unit</t>
+  </si>
+  <si>
+    <t>COD</t>
+  </si>
+  <si>
+    <t>TN</t>
+  </si>
+  <si>
+    <t>TP</t>
+  </si>
+  <si>
+    <t>TSS</t>
   </si>
   <si>
     <t>Dissolved</t>
@@ -2159,33 +2171,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:W21"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="6.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.08984375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="3.26953125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5.7265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="3.36328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="3.7265625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="4.08984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="6.36328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="4.81640625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="6.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="6.54296875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="4" width="12" customWidth="1"/>
+    <col min="5" max="7" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>50</v>
       </c>
@@ -2195,1484 +2190,404 @@
       <c r="C1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>15</v>
-      </c>
-      <c r="R1" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" t="s">
-        <v>17</v>
-      </c>
-      <c r="T1" t="s">
-        <v>18</v>
-      </c>
-      <c r="U1" t="s">
-        <v>19</v>
-      </c>
-      <c r="V1" t="s">
-        <v>20</v>
-      </c>
-      <c r="W1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="D1" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-      <c r="P2">
-        <v>0</v>
-      </c>
-      <c r="Q2">
-        <v>0</v>
-      </c>
-      <c r="R2">
-        <v>0</v>
-      </c>
-      <c r="S2">
-        <v>0</v>
-      </c>
-      <c r="T2">
-        <v>0</v>
-      </c>
-      <c r="U2">
-        <v>0</v>
-      </c>
-      <c r="V2">
-        <v>0</v>
-      </c>
-      <c r="W2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D3">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <f>parameter_table!$E$11</f>
         <v>0</v>
       </c>
-      <c r="E3">
-        <v>1</v>
-      </c>
       <c r="F3">
+        <f>parameter_table!$E$16</f>
         <v>0</v>
       </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-      <c r="L3">
-        <v>0</v>
-      </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
-      <c r="N3">
-        <v>0</v>
-      </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="P3">
-        <v>0</v>
-      </c>
-      <c r="Q3">
-        <v>0</v>
-      </c>
-      <c r="R3">
-        <v>0</v>
-      </c>
-      <c r="S3">
-        <v>0</v>
-      </c>
-      <c r="T3">
-        <v>0</v>
-      </c>
-      <c r="U3">
-        <v>0</v>
-      </c>
-      <c r="V3">
-        <v>0</v>
-      </c>
-      <c r="W3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B4" t="s">
         <v>4</v>
       </c>
       <c r="C4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
+        <f>1</f>
         <v>1</v>
       </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>0</v>
-      </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="P4">
-        <v>0</v>
-      </c>
-      <c r="Q4">
-        <v>0</v>
-      </c>
-      <c r="R4">
-        <v>0</v>
-      </c>
-      <c r="S4">
-        <v>0</v>
-      </c>
-      <c r="T4">
-        <v>0</v>
-      </c>
-      <c r="U4">
-        <v>0</v>
-      </c>
-      <c r="V4">
-        <v>0</v>
-      </c>
-      <c r="W4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.35">
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>56</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
+        <f>1</f>
         <v>1</v>
       </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5">
-        <v>0</v>
-      </c>
-      <c r="K5">
-        <v>0</v>
-      </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="N5">
-        <v>0</v>
-      </c>
-      <c r="O5">
-        <v>0</v>
-      </c>
-      <c r="P5">
-        <v>0</v>
-      </c>
-      <c r="Q5">
-        <v>0</v>
-      </c>
-      <c r="R5">
-        <v>0</v>
-      </c>
-      <c r="S5">
-        <v>0</v>
-      </c>
-      <c r="T5">
-        <v>0</v>
-      </c>
-      <c r="U5">
-        <v>0</v>
-      </c>
-      <c r="V5">
-        <v>0</v>
-      </c>
-      <c r="W5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
+        <f>1</f>
         <v>1</v>
       </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6">
-        <v>0</v>
-      </c>
-      <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="N6">
-        <v>0</v>
-      </c>
-      <c r="O6">
-        <v>0</v>
-      </c>
-      <c r="P6">
-        <v>0</v>
-      </c>
-      <c r="Q6">
-        <v>0</v>
-      </c>
-      <c r="R6">
-        <v>0</v>
-      </c>
-      <c r="S6">
-        <v>0</v>
-      </c>
-      <c r="T6">
-        <v>0</v>
-      </c>
-      <c r="U6">
-        <v>0</v>
-      </c>
-      <c r="V6">
-        <v>0</v>
-      </c>
-      <c r="W6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B7" t="s">
         <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
+        <f>1</f>
         <v>1</v>
       </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7">
-        <v>0</v>
-      </c>
-      <c r="O7">
-        <v>0</v>
-      </c>
-      <c r="P7">
-        <v>0</v>
-      </c>
-      <c r="Q7">
-        <v>0</v>
-      </c>
-      <c r="R7">
-        <v>0</v>
-      </c>
-      <c r="S7">
-        <v>0</v>
-      </c>
-      <c r="T7">
-        <v>0</v>
-      </c>
-      <c r="U7">
-        <v>0</v>
-      </c>
-      <c r="V7">
-        <v>0</v>
-      </c>
-      <c r="W7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B8" t="s">
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>56</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8">
-        <v>1</v>
-      </c>
-      <c r="K8">
-        <v>0</v>
-      </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8">
-        <v>0</v>
-      </c>
-      <c r="N8">
-        <v>0</v>
-      </c>
-      <c r="O8">
-        <v>0</v>
-      </c>
-      <c r="P8">
-        <v>0</v>
-      </c>
-      <c r="Q8">
-        <v>0</v>
-      </c>
-      <c r="R8">
-        <v>0</v>
-      </c>
-      <c r="S8">
-        <v>0</v>
-      </c>
-      <c r="T8">
-        <v>0</v>
-      </c>
-      <c r="U8">
-        <v>0</v>
-      </c>
-      <c r="V8">
-        <v>0</v>
-      </c>
-      <c r="W8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s">
         <v>9</v>
       </c>
       <c r="C9" t="s">
+        <v>61</v>
+      </c>
+      <c r="F9">
+        <f>1</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>57</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9">
-        <v>1</v>
-      </c>
-      <c r="L9">
-        <v>0</v>
-      </c>
-      <c r="M9">
-        <v>0</v>
-      </c>
-      <c r="N9">
-        <v>0</v>
-      </c>
-      <c r="O9">
-        <v>0</v>
-      </c>
-      <c r="P9">
-        <v>0</v>
-      </c>
-      <c r="Q9">
-        <v>0</v>
-      </c>
-      <c r="R9">
-        <v>0</v>
-      </c>
-      <c r="S9">
-        <v>0</v>
-      </c>
-      <c r="T9">
-        <v>0</v>
-      </c>
-      <c r="U9">
-        <v>0</v>
-      </c>
-      <c r="V9">
-        <v>0</v>
-      </c>
-      <c r="W9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>53</v>
       </c>
       <c r="B10" t="s">
         <v>10</v>
       </c>
       <c r="C10" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D10">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <f>parameter_table!$E$10</f>
+        <v>0.01</v>
+      </c>
+      <c r="F10">
+        <f>parameter_table!$E$15</f>
         <v>0</v>
       </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-      <c r="H10">
-        <v>0</v>
-      </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
-      <c r="J10">
-        <v>0</v>
-      </c>
-      <c r="K10">
-        <v>0</v>
-      </c>
-      <c r="L10">
-        <v>1</v>
-      </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
-      <c r="N10">
-        <v>0</v>
-      </c>
-      <c r="O10">
-        <v>0</v>
-      </c>
-      <c r="P10">
-        <v>0</v>
-      </c>
-      <c r="Q10">
-        <v>0</v>
-      </c>
-      <c r="R10">
-        <v>0</v>
-      </c>
-      <c r="S10">
-        <v>0</v>
-      </c>
-      <c r="T10">
-        <v>0</v>
-      </c>
-      <c r="U10">
-        <v>0</v>
-      </c>
-      <c r="V10">
-        <v>0</v>
-      </c>
-      <c r="W10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
         <v>11</v>
       </c>
       <c r="C11" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-      <c r="H11">
-        <v>0</v>
-      </c>
-      <c r="I11">
-        <v>0</v>
-      </c>
-      <c r="J11">
-        <v>0</v>
-      </c>
-      <c r="K11">
-        <v>0</v>
-      </c>
-      <c r="L11">
-        <v>0</v>
-      </c>
-      <c r="M11">
-        <v>1</v>
-      </c>
-      <c r="N11">
-        <v>0</v>
-      </c>
-      <c r="O11">
-        <v>0</v>
-      </c>
-      <c r="P11">
-        <v>0</v>
-      </c>
-      <c r="Q11">
-        <v>0</v>
-      </c>
-      <c r="R11">
-        <v>0</v>
-      </c>
-      <c r="S11">
-        <v>0</v>
-      </c>
-      <c r="T11">
-        <v>0</v>
-      </c>
-      <c r="U11">
-        <v>0</v>
-      </c>
-      <c r="V11">
-        <v>0</v>
-      </c>
-      <c r="W11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B12" t="s">
         <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <f>1</f>
+        <v>1</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <f>parameter_table!$E$12</f>
+        <v>0.02</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <f>parameter_table!$E$17</f>
+        <v>0.01</v>
       </c>
       <c r="G12">
-        <v>0</v>
-      </c>
-      <c r="H12">
-        <v>0</v>
-      </c>
-      <c r="I12">
-        <v>0</v>
-      </c>
-      <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="N12">
-        <v>1</v>
-      </c>
-      <c r="O12">
-        <v>0</v>
-      </c>
-      <c r="P12">
-        <v>0</v>
-      </c>
-      <c r="Q12">
-        <v>0</v>
-      </c>
-      <c r="R12">
-        <v>0</v>
-      </c>
-      <c r="S12">
-        <v>0</v>
-      </c>
-      <c r="T12">
-        <v>0</v>
-      </c>
-      <c r="U12">
-        <v>0</v>
-      </c>
-      <c r="V12">
-        <v>0</v>
-      </c>
-      <c r="W12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+        <f>parameter_table!$E$20</f>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B13" t="s">
         <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D13">
+        <f>1</f>
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <f>parameter_table!$E$13</f>
         <v>0</v>
       </c>
-      <c r="E13">
+      <c r="F13">
+        <f>parameter_table!$E$18</f>
         <v>0</v>
       </c>
-      <c r="F13">
-        <v>0</v>
-      </c>
       <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
-      <c r="I13">
-        <v>0</v>
-      </c>
-      <c r="J13">
-        <v>0</v>
-      </c>
-      <c r="K13">
-        <v>0</v>
-      </c>
-      <c r="L13">
-        <v>0</v>
-      </c>
-      <c r="M13">
-        <v>0</v>
-      </c>
-      <c r="N13">
-        <v>0</v>
-      </c>
-      <c r="O13">
-        <v>1</v>
-      </c>
-      <c r="P13">
-        <v>0</v>
-      </c>
-      <c r="Q13">
-        <v>0</v>
-      </c>
-      <c r="R13">
-        <v>0</v>
-      </c>
-      <c r="S13">
-        <v>0</v>
-      </c>
-      <c r="T13">
-        <v>0</v>
-      </c>
-      <c r="U13">
-        <v>0</v>
-      </c>
-      <c r="V13">
-        <v>0</v>
-      </c>
-      <c r="W13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
+        <f>parameter_table!$E$21</f>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B14" t="s">
         <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D14">
-        <v>0</v>
+        <f>1</f>
+        <v>1</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <f>parameter_table!$E$14</f>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <f>parameter_table!$E$19</f>
+        <v>0.02</v>
       </c>
       <c r="G14">
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <v>0</v>
-      </c>
-      <c r="I14">
-        <v>0</v>
-      </c>
-      <c r="J14">
-        <v>0</v>
-      </c>
-      <c r="K14">
-        <v>0</v>
-      </c>
-      <c r="L14">
-        <v>0</v>
-      </c>
-      <c r="M14">
-        <v>0</v>
-      </c>
-      <c r="N14">
-        <v>0</v>
-      </c>
-      <c r="O14">
-        <v>0</v>
-      </c>
-      <c r="P14">
-        <v>1</v>
-      </c>
-      <c r="Q14">
-        <v>0</v>
-      </c>
-      <c r="R14">
-        <v>0</v>
-      </c>
-      <c r="S14">
-        <v>0</v>
-      </c>
-      <c r="T14">
-        <v>0</v>
-      </c>
-      <c r="U14">
-        <v>0</v>
-      </c>
-      <c r="V14">
-        <v>0</v>
-      </c>
-      <c r="W14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
+        <f>parameter_table!$E$22</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B15" t="s">
         <v>15</v>
       </c>
       <c r="C15" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <f>1</f>
+        <v>1</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <f>parameter_table!$E$14</f>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <f>parameter_table!$E$19</f>
+        <v>0.02</v>
       </c>
       <c r="G15">
-        <v>0</v>
-      </c>
-      <c r="H15">
-        <v>0</v>
-      </c>
-      <c r="I15">
-        <v>0</v>
-      </c>
-      <c r="J15">
-        <v>0</v>
-      </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15">
-        <v>0</v>
-      </c>
-      <c r="M15">
-        <v>0</v>
-      </c>
-      <c r="N15">
-        <v>0</v>
-      </c>
-      <c r="O15">
-        <v>0</v>
-      </c>
-      <c r="P15">
-        <v>0</v>
-      </c>
-      <c r="Q15">
-        <v>1</v>
-      </c>
-      <c r="R15">
-        <v>0</v>
-      </c>
-      <c r="S15">
-        <v>0</v>
-      </c>
-      <c r="T15">
-        <v>0</v>
-      </c>
-      <c r="U15">
-        <v>0</v>
-      </c>
-      <c r="V15">
-        <v>0</v>
-      </c>
-      <c r="W15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+        <f>parameter_table!$E$22</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B16" t="s">
         <v>16</v>
       </c>
       <c r="C16" t="s">
-        <v>57</v>
-      </c>
-      <c r="D16">
-        <v>0</v>
-      </c>
-      <c r="E16">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="F16">
-        <v>0</v>
+        <f>1</f>
+        <v>1</v>
       </c>
       <c r="G16">
-        <v>0</v>
-      </c>
-      <c r="H16">
-        <v>0</v>
-      </c>
-      <c r="I16">
-        <v>0</v>
-      </c>
-      <c r="J16">
-        <v>0</v>
-      </c>
-      <c r="K16">
-        <v>0</v>
-      </c>
-      <c r="L16">
-        <v>0</v>
-      </c>
-      <c r="M16">
-        <v>0</v>
-      </c>
-      <c r="N16">
-        <v>0</v>
-      </c>
-      <c r="O16">
-        <v>0</v>
-      </c>
-      <c r="P16">
-        <v>0</v>
-      </c>
-      <c r="Q16">
-        <v>0</v>
-      </c>
-      <c r="R16">
-        <v>1</v>
-      </c>
-      <c r="S16">
-        <v>0</v>
-      </c>
-      <c r="T16">
-        <v>0</v>
-      </c>
-      <c r="U16">
-        <v>0</v>
-      </c>
-      <c r="V16">
-        <v>0</v>
-      </c>
-      <c r="W16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+        <f>parameter_table!$E$24</f>
+        <v>3.23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B17" t="s">
         <v>17</v>
       </c>
       <c r="C17" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D17">
-        <v>0</v>
-      </c>
-      <c r="E17">
-        <v>0</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
+        <f>1</f>
+        <v>1</v>
       </c>
       <c r="G17">
-        <v>0</v>
-      </c>
-      <c r="H17">
-        <v>0</v>
-      </c>
-      <c r="I17">
-        <v>0</v>
-      </c>
-      <c r="J17">
-        <v>0</v>
-      </c>
-      <c r="K17">
-        <v>0</v>
-      </c>
-      <c r="L17">
-        <v>0</v>
-      </c>
-      <c r="M17">
-        <v>0</v>
-      </c>
-      <c r="N17">
-        <v>0</v>
-      </c>
-      <c r="O17">
-        <v>0</v>
-      </c>
-      <c r="P17">
-        <v>0</v>
-      </c>
-      <c r="Q17">
-        <v>0</v>
-      </c>
-      <c r="R17">
-        <v>0</v>
-      </c>
-      <c r="S17">
-        <v>1</v>
-      </c>
-      <c r="T17">
-        <v>0</v>
-      </c>
-      <c r="U17">
-        <v>0</v>
-      </c>
-      <c r="V17">
-        <v>0</v>
-      </c>
-      <c r="W17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+        <f>parameter_table!$E$23</f>
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B18" t="s">
         <v>18</v>
       </c>
       <c r="C18" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D18">
-        <v>0</v>
+        <f>1</f>
+        <v>1</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <f>parameter_table!$E$14</f>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <f>parameter_table!$E$19</f>
+        <v>0.02</v>
       </c>
       <c r="G18">
-        <v>0</v>
-      </c>
-      <c r="H18">
-        <v>0</v>
-      </c>
-      <c r="I18">
-        <v>0</v>
-      </c>
-      <c r="J18">
-        <v>0</v>
-      </c>
-      <c r="K18">
-        <v>0</v>
-      </c>
-      <c r="L18">
-        <v>0</v>
-      </c>
-      <c r="M18">
-        <v>0</v>
-      </c>
-      <c r="N18">
-        <v>0</v>
-      </c>
-      <c r="O18">
-        <v>0</v>
-      </c>
-      <c r="P18">
-        <v>0</v>
-      </c>
-      <c r="Q18">
-        <v>0</v>
-      </c>
-      <c r="R18">
-        <v>0</v>
-      </c>
-      <c r="S18">
-        <v>0</v>
-      </c>
-      <c r="T18">
-        <v>1</v>
-      </c>
-      <c r="U18">
-        <v>0</v>
-      </c>
-      <c r="V18">
-        <v>0</v>
-      </c>
-      <c r="W18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
+        <f>parameter_table!$E$22</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B19" t="s">
         <v>19</v>
       </c>
       <c r="C19" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D19">
-        <v>0</v>
+        <f>1</f>
+        <v>1</v>
       </c>
       <c r="E19">
-        <v>0</v>
+        <f>parameter_table!$E$14</f>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <f>parameter_table!$E$19</f>
+        <v>0.02</v>
       </c>
       <c r="G19">
-        <v>0</v>
-      </c>
-      <c r="H19">
-        <v>0</v>
-      </c>
-      <c r="I19">
-        <v>0</v>
-      </c>
-      <c r="J19">
-        <v>0</v>
-      </c>
-      <c r="K19">
-        <v>0</v>
-      </c>
-      <c r="L19">
-        <v>0</v>
-      </c>
-      <c r="M19">
-        <v>0</v>
-      </c>
-      <c r="N19">
-        <v>0</v>
-      </c>
-      <c r="O19">
-        <v>0</v>
-      </c>
-      <c r="P19">
-        <v>0</v>
-      </c>
-      <c r="Q19">
-        <v>0</v>
-      </c>
-      <c r="R19">
-        <v>0</v>
-      </c>
-      <c r="S19">
-        <v>0</v>
-      </c>
-      <c r="T19">
-        <v>0</v>
-      </c>
-      <c r="U19">
-        <v>1</v>
-      </c>
-      <c r="V19">
-        <v>0</v>
-      </c>
-      <c r="W19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.35">
+        <f>parameter_table!$E$22</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B20" t="s">
         <v>20</v>
       </c>
       <c r="C20" t="s">
-        <v>60</v>
-      </c>
-      <c r="D20">
-        <v>0</v>
-      </c>
-      <c r="E20">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="F20">
-        <v>0</v>
+        <f>parameter_table!$E$25</f>
+        <v>0.20499999999999999</v>
       </c>
       <c r="G20">
-        <v>0</v>
-      </c>
-      <c r="H20">
-        <v>0</v>
-      </c>
-      <c r="I20">
-        <v>0</v>
-      </c>
-      <c r="J20">
-        <v>0</v>
-      </c>
-      <c r="K20">
-        <v>0</v>
-      </c>
-      <c r="L20">
-        <v>0</v>
-      </c>
-      <c r="M20">
-        <v>0</v>
-      </c>
-      <c r="N20">
-        <v>0</v>
-      </c>
-      <c r="O20">
-        <v>0</v>
-      </c>
-      <c r="P20">
-        <v>0</v>
-      </c>
-      <c r="Q20">
-        <v>0</v>
-      </c>
-      <c r="R20">
-        <v>0</v>
-      </c>
-      <c r="S20">
-        <v>0</v>
-      </c>
-      <c r="T20">
-        <v>0</v>
-      </c>
-      <c r="U20">
-        <v>0</v>
-      </c>
-      <c r="V20">
+        <f>1</f>
         <v>1</v>
       </c>
-      <c r="W20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B21" t="s">
         <v>21</v>
       </c>
       <c r="C21" t="s">
-        <v>60</v>
-      </c>
-      <c r="D21">
-        <v>0</v>
-      </c>
-      <c r="E21">
-        <v>0</v>
-      </c>
-      <c r="F21">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="G21">
-        <v>0</v>
-      </c>
-      <c r="H21">
-        <v>0</v>
-      </c>
-      <c r="I21">
-        <v>0</v>
-      </c>
-      <c r="J21">
-        <v>0</v>
-      </c>
-      <c r="K21">
-        <v>0</v>
-      </c>
-      <c r="L21">
-        <v>0</v>
-      </c>
-      <c r="M21">
-        <v>0</v>
-      </c>
-      <c r="N21">
-        <v>0</v>
-      </c>
-      <c r="O21">
-        <v>0</v>
-      </c>
-      <c r="P21">
-        <v>0</v>
-      </c>
-      <c r="Q21">
-        <v>0</v>
-      </c>
-      <c r="R21">
-        <v>0</v>
-      </c>
-      <c r="S21">
-        <v>0</v>
-      </c>
-      <c r="T21">
-        <v>0</v>
-      </c>
-      <c r="U21">
-        <v>0</v>
-      </c>
-      <c r="V21">
-        <v>0</v>
-      </c>
-      <c r="W21">
+        <f>1</f>
         <v>1</v>
       </c>
     </row>
@@ -3699,19 +2614,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>52</v>
@@ -3719,1622 +2634,1622 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E2" s="3">
         <v>0.625</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E3" s="4">
         <v>0.625</v>
       </c>
       <c r="F3" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C4" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D4" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E4" s="4">
         <v>0.2</v>
       </c>
       <c r="F4" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B5" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C5" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D5" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E5" s="4">
         <v>0.4</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B6" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D6" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="E6" s="4">
         <v>0.18</v>
       </c>
       <c r="F6" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B7" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C7" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D7" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E7" s="4">
         <v>0.08</v>
       </c>
       <c r="F7" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C8" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D8" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E8" s="4">
         <v>0</v>
       </c>
       <c r="F8" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B9" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C9" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D9" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="E9" s="4">
         <v>0.1</v>
       </c>
       <c r="F9" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="E10" s="3">
         <v>0.01</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B11" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C11" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D11" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="E11" s="4">
         <v>0</v>
       </c>
       <c r="F11" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B12" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C12" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D12" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="E12" s="4">
         <v>0.02</v>
       </c>
       <c r="F12" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B13" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C13" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D13" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="E13" s="4">
         <v>0</v>
       </c>
       <c r="F13" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B14" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C14" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D14" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="E14" s="4">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F14" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B15" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C15" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D15" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="E15" s="4">
         <v>0</v>
       </c>
       <c r="F15" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B16" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C16" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="D16" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="E16" s="4">
         <v>0</v>
       </c>
       <c r="F16" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B17" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C17" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D17" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="E17" s="4">
         <v>0.01</v>
       </c>
       <c r="F17" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B18" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C18" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D18" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="E18" s="4">
         <v>0</v>
       </c>
       <c r="F18" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C19" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D19" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E19" s="4">
         <v>0.02</v>
       </c>
       <c r="F19" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B20" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C20" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D20" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="E20" s="4">
         <v>0.75</v>
       </c>
       <c r="F20" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B21" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C21" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D21" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="E21" s="4">
         <v>0.75</v>
       </c>
       <c r="F21" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B22" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C22" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D22" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="E22" s="4">
         <v>0.9</v>
       </c>
       <c r="F22" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B23" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C23" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D23" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="E23" s="4">
         <v>0.6</v>
       </c>
       <c r="F23" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B24" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C24" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D24" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="E24" s="4">
         <v>3.23</v>
       </c>
       <c r="F24" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B25" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C25" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D25" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="E25" s="4">
         <v>0.20499999999999999</v>
       </c>
       <c r="F25" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="E26" s="3">
         <v>3</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B27" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C27" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D27" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="E27" s="4">
         <v>0.6</v>
       </c>
       <c r="F27" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B28" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C28" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D28" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E28" s="4">
         <v>0.6</v>
       </c>
       <c r="F28" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B29" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C29" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="D29" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E29" s="4">
         <v>0.4</v>
       </c>
       <c r="F29" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B30" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="C30" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D30" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="E30" s="4">
         <v>0.2</v>
       </c>
       <c r="F30" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B31" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C31" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D31" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="E31" s="4">
         <v>0.5</v>
       </c>
       <c r="F31" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B32" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C32" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="D32" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="E32" s="4">
         <v>0.5</v>
       </c>
       <c r="F32" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B33" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C33" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D33" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="E33" s="4">
         <v>0.5</v>
       </c>
       <c r="F33" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B34" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C34" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="D34" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="E34" s="4">
         <v>0.1</v>
       </c>
       <c r="F34" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E35" s="3">
         <v>6</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B36" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="C36" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D36" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="E36" s="4">
         <v>3</v>
       </c>
       <c r="F36" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B37" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C37" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D37" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="E37" s="4">
         <v>0.9</v>
       </c>
       <c r="F37" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B38" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C38" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D38" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="E38" s="4">
         <v>0.9</v>
       </c>
       <c r="F38" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B39" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="C39" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D39" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="E39" s="4">
         <v>0.4</v>
       </c>
       <c r="F39" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B40" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C40" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="D40" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="E40" s="4">
         <v>0.2</v>
       </c>
       <c r="F40" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B41" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C41" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="D41" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="E41" s="4">
         <v>4</v>
       </c>
       <c r="F41" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B42" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C42" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="D42" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="E42" s="4">
         <v>4</v>
       </c>
       <c r="F42" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B43" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="C43" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D43" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E43" s="4">
         <v>4</v>
       </c>
       <c r="F43" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B44" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="C44" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="D44" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="E44" s="4">
         <v>0.5</v>
       </c>
       <c r="F44" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B45" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C45" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="D45" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="E45" s="4">
         <v>0.5</v>
       </c>
       <c r="F45" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B46" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="C46" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="D46" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="E46" s="4">
         <v>0.5</v>
       </c>
       <c r="F46" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B47" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="C47" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="D47" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="E47" s="4">
         <v>0.05</v>
       </c>
       <c r="F47" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B48" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C48" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="D48" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="E48" s="4">
         <v>0.01</v>
       </c>
       <c r="F48" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B49" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C49" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="D49" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="E49" s="4">
         <v>0.1</v>
       </c>
       <c r="F49" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="E50" s="3">
         <v>5</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B51" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C51" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="D51" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="E51" s="4">
         <v>0.6</v>
       </c>
       <c r="F51" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B52" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C52" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="D52" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="E52" s="4">
         <v>0.56000000000000005</v>
       </c>
       <c r="F52" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B53" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C53" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="D53" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="E53" s="4">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F53" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B54" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C54" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="D54" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="E54" s="4">
         <v>0.9</v>
       </c>
       <c r="F54" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B55" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C55" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D55" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="E55" s="4">
         <v>0.2</v>
       </c>
       <c r="F55" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B56" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C56" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="D56" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="E56" s="4">
         <v>0.2</v>
       </c>
       <c r="F56" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B57" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C57" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="D57" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="E57" s="4">
         <v>0.2</v>
       </c>
       <c r="F57" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B58" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C58" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="D58" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="E58" s="4">
         <v>0.2</v>
       </c>
       <c r="F58" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B59" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C59" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="D59" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="E59" s="4">
         <v>0.5</v>
       </c>
       <c r="F59" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B60" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C60" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="D60" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="E60" s="4">
         <v>0.5</v>
       </c>
       <c r="F60" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B61" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C61" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="D61" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="E61" s="4">
         <v>0.5</v>
       </c>
       <c r="F61" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B62" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C62" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="D62" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="E62" s="4">
         <v>0.05</v>
       </c>
       <c r="F62" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B63" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C63" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="D63" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="E63" s="4">
         <v>0.2</v>
       </c>
       <c r="F63" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B64" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C64" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="D64" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="E64" s="4">
         <v>0.01</v>
       </c>
       <c r="F64" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B65" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="C65" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="D65" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="E65" s="4">
         <v>0.1</v>
       </c>
       <c r="F65" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B66" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="C66" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="D66" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="E66" s="4">
         <v>0.01</v>
       </c>
       <c r="F66" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B67" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="C67" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D67" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E67" s="4">
         <v>0.34</v>
       </c>
       <c r="F67" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B68" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="C68" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="D68" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="E68" s="4">
         <v>0.02</v>
       </c>
       <c r="F68" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B69" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="C69" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D69" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E69" s="4">
         <v>0.01</v>
       </c>
       <c r="F69" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="D70" s="2" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="E70" s="3">
         <v>1.81</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B71" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="C71" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="D71" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="E71" s="4">
         <v>1.52</v>
       </c>
       <c r="F71" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B72" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="C72" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="D72" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="E72" s="4">
         <v>0.2</v>
       </c>
       <c r="F72" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B73" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="C73" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="D73" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E73" s="4">
         <v>0.17</v>
       </c>
       <c r="F73" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B74" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="C74" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="D74" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="E74" s="4">
         <v>0.74</v>
       </c>
       <c r="F74" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B75" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="C75" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="D75" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E75" s="4">
         <v>1.75</v>
       </c>
       <c r="F75" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B76" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="C76" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="D76" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E76" s="4">
         <v>0.5</v>
       </c>
       <c r="F76" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B77" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C77" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="D77" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="E77" s="4">
         <v>0.5</v>
       </c>
       <c r="F77" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B78" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C78" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="D78" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="E78" s="4">
         <v>0.5</v>
       </c>
       <c r="F78" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B79" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C79" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="D79" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="E79" s="4">
         <v>0.01</v>
       </c>
       <c r="F79" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="E80" s="3">
         <v>1</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B81" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C81" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="D81" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="E81" s="4">
         <v>0.6</v>
       </c>
       <c r="F81" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B82" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C82" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="D82" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="E82" s="4">
         <v>0.5</v>
       </c>
       <c r="F82" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>